<commit_message>
#159 Bottom Board BOM Updated
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark-BOM-Bottom (20 Board).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark-BOM-Bottom (20 Board).xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F0F123-5582-4C09-B5D2-11D3E2F71EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -129,9 +143,6 @@
     <t>U5</t>
   </si>
   <si>
-    <t>U9</t>
-  </si>
-  <si>
     <t>U10</t>
   </si>
   <si>
@@ -685,12 +696,15 @@
   </si>
   <si>
     <t>Multiple options added for MCU</t>
+  </si>
+  <si>
+    <t>U6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1829,7 +1843,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1882,7 +1896,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="56" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1906,7 +1920,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="57" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1930,7 +1944,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="58" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -2035,52 +2049,52 @@
         <v>4</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D9" s="30" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="61" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H9" s="60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="K9" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="M9" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="J9" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>209</v>
-      </c>
-      <c r="L9" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="M9" s="30" t="s">
+      <c r="N9" s="60" t="s">
         <v>159</v>
       </c>
-      <c r="N9" s="60" t="s">
+      <c r="O9" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="O9" s="30" t="s">
+      <c r="P9" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="P9" s="30" t="s">
+      <c r="Q9" s="60" t="s">
         <v>162</v>
       </c>
-      <c r="Q9" s="60" t="s">
+      <c r="R9" s="30" t="s">
         <v>163</v>
-      </c>
-      <c r="R9" s="30" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -2090,31 +2104,31 @@
         <v>1</v>
       </c>
       <c r="C10" s="92" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D10" s="93" t="s">
         <v>9</v>
       </c>
       <c r="E10" s="93" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" s="94" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G10" s="93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H10" s="94" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I10" s="93" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J10" s="94" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K10" s="93" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L10" s="95">
         <v>1</v>
@@ -2127,7 +2141,7 @@
         <v>40</v>
       </c>
       <c r="O10" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P10" s="96">
         <v>1.7399999999999999E-2</v>
@@ -2145,31 +2159,31 @@
         <v>2</v>
       </c>
       <c r="C11" s="85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D11" s="86" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E11" s="86" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G11" s="86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H11" s="87" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I11" s="86" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J11" s="87" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K11" s="86" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="L11" s="89">
         <v>18</v>
@@ -2182,7 +2196,7 @@
         <v>400</v>
       </c>
       <c r="O11" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P11" s="90">
         <v>2.3999999999999998E-3</v>
@@ -2200,31 +2214,31 @@
         <v>3</v>
       </c>
       <c r="C12" s="92" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D12" s="93" t="s">
         <v>10</v>
       </c>
       <c r="E12" s="93" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F12" s="94" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G12" s="93" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H12" s="94" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I12" s="93" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J12" s="94" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K12" s="93" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L12" s="95">
         <v>1</v>
@@ -2237,7 +2251,7 @@
         <v>25</v>
       </c>
       <c r="O12" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P12" s="96">
         <v>5.2600000000000001E-2</v>
@@ -2255,31 +2269,31 @@
         <v>4</v>
       </c>
       <c r="C13" s="85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D13" s="86" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="86" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F13" s="87" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G13" s="86" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H13" s="87" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I13" s="86" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J13" s="87" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K13" s="86" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="L13" s="89">
         <v>2</v>
@@ -2292,7 +2306,7 @@
         <v>50</v>
       </c>
       <c r="O13" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P13" s="90">
         <v>5.96E-2</v>
@@ -2310,31 +2324,31 @@
         <v>5</v>
       </c>
       <c r="C14" s="92" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D14" s="93" t="s">
         <v>12</v>
       </c>
       <c r="E14" s="93" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F14" s="94" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G14" s="93" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H14" s="94" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I14" s="93" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J14" s="94" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K14" s="93" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L14" s="95">
         <v>2</v>
@@ -2347,7 +2361,7 @@
         <v>100</v>
       </c>
       <c r="O14" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P14" s="96">
         <v>2.5999999999999999E-3</v>
@@ -2365,31 +2379,31 @@
         <v>6</v>
       </c>
       <c r="C15" s="85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" s="86" t="s">
         <v>13</v>
       </c>
       <c r="E15" s="86" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F15" s="87" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G15" s="88" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H15" s="87" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I15" s="86" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J15" s="87" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K15" s="86" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L15" s="89">
         <v>2</v>
@@ -2402,7 +2416,7 @@
         <v>50</v>
       </c>
       <c r="O15" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P15" s="90">
         <v>6.4000000000000003E-3</v>
@@ -2420,31 +2434,31 @@
         <v>7</v>
       </c>
       <c r="C16" s="64" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D16" s="40" t="s">
         <v>14</v>
       </c>
       <c r="E16" s="40" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G16" s="77" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H16" s="41" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I16" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J16" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K16" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L16" s="79">
         <v>1</v>
@@ -2457,7 +2471,7 @@
         <v>25</v>
       </c>
       <c r="O16" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P16" s="53">
         <v>0.1772</v>
@@ -2475,31 +2489,31 @@
         <v>8</v>
       </c>
       <c r="C17" s="65" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D17" s="38" t="s">
         <v>15</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G17" s="38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K17" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L17" s="78">
         <v>1</v>
@@ -2512,7 +2526,7 @@
         <v>25</v>
       </c>
       <c r="O17" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P17" s="52">
         <v>6.1699999999999998E-2</v>
@@ -2530,31 +2544,31 @@
         <v>9</v>
       </c>
       <c r="C18" s="64" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D18" s="40" t="s">
         <v>16</v>
       </c>
       <c r="E18" s="40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F18" s="41" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G18" s="40" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H18" s="41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I18" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J18" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K18" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L18" s="79">
         <v>4</v>
@@ -2567,7 +2581,7 @@
         <v>100</v>
       </c>
       <c r="O18" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P18" s="53">
         <v>2.8000000000000001E-2</v>
@@ -2585,31 +2599,31 @@
         <v>10</v>
       </c>
       <c r="C19" s="63" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D19" s="38" t="s">
         <v>17</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F19" s="39" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G19" s="38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L19" s="78">
         <v>1</v>
@@ -2622,7 +2636,7 @@
         <v>22</v>
       </c>
       <c r="O19" s="74" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P19" s="52">
         <v>2.5099999999999998</v>
@@ -2640,31 +2654,31 @@
         <v>11</v>
       </c>
       <c r="C20" s="64" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D20" s="40" t="s">
         <v>18</v>
       </c>
       <c r="E20" s="40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F20" s="41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G20" s="40" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H20" s="41" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I20" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J20" s="41" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K20" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L20" s="79">
         <v>1</v>
@@ -2677,7 +2691,7 @@
         <v>25</v>
       </c>
       <c r="O20" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P20" s="53">
         <v>8.7599999999999997E-2</v>
@@ -2695,31 +2709,31 @@
         <v>12</v>
       </c>
       <c r="C21" s="63" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D21" s="38" t="s">
         <v>19</v>
       </c>
       <c r="E21" s="38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F21" s="39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G21" s="67" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K21" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L21" s="78">
         <v>1</v>
@@ -2732,7 +2746,7 @@
         <v>30</v>
       </c>
       <c r="O21" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P21" s="52">
         <v>3.7900000000000003E-2</v>
@@ -2750,31 +2764,31 @@
         <v>13</v>
       </c>
       <c r="C22" s="64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D22" s="40" t="s">
         <v>20</v>
       </c>
       <c r="E22" s="40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F22" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G22" s="40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H22" s="41" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I22" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J22" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K22" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L22" s="79">
         <v>1</v>
@@ -2787,7 +2801,7 @@
         <v>25</v>
       </c>
       <c r="O22" s="73" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="P22" s="53">
         <v>0.30840000000000001</v>
@@ -2805,31 +2819,31 @@
         <v>14</v>
       </c>
       <c r="C23" s="63" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D23" s="38" t="s">
         <v>21</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F23" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J23" s="39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K23" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L23" s="78">
         <v>2</v>
@@ -2842,7 +2856,7 @@
         <v>60</v>
       </c>
       <c r="O23" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P23" s="52">
         <v>3.0599999999999999E-2</v>
@@ -2860,31 +2874,31 @@
         <v>15</v>
       </c>
       <c r="C24" s="64" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D24" s="40" t="s">
         <v>22</v>
       </c>
       <c r="E24" s="40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F24" s="41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G24" s="40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H24" s="41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I24" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J24" s="41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K24" s="40" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="L24" s="79">
         <v>40</v>
@@ -2897,7 +2911,7 @@
         <v>900</v>
       </c>
       <c r="O24" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P24" s="53">
         <v>8.0000000000000004E-4</v>
@@ -2915,31 +2929,31 @@
         <v>16</v>
       </c>
       <c r="C25" s="63" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D25" s="38" t="s">
         <v>23</v>
       </c>
       <c r="E25" s="38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J25" s="39" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K25" s="38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L25" s="78">
         <v>7</v>
@@ -2952,7 +2966,7 @@
         <v>200</v>
       </c>
       <c r="O25" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P25" s="52">
         <v>1E-3</v>
@@ -2970,31 +2984,31 @@
         <v>17</v>
       </c>
       <c r="C26" s="64" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D26" s="40" t="s">
         <v>24</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F26" s="41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G26" s="76" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H26" s="41" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J26" s="41" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K26" s="40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L26" s="79">
         <v>1</v>
@@ -3007,7 +3021,7 @@
         <v>100</v>
       </c>
       <c r="O26" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P26" s="53">
         <v>1.9E-3</v>
@@ -3025,31 +3039,31 @@
         <v>18</v>
       </c>
       <c r="C27" s="63" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D27" s="38" t="s">
         <v>25</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G27" s="38" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H27" s="39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J27" s="39" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K27" s="38" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="L27" s="78">
         <v>2</v>
@@ -3062,7 +3076,7 @@
         <v>100</v>
       </c>
       <c r="O27" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P27" s="52">
         <v>1E-3</v>
@@ -3080,31 +3094,31 @@
         <v>19</v>
       </c>
       <c r="C28" s="64" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D28" s="40" t="s">
         <v>26</v>
       </c>
       <c r="E28" s="40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F28" s="41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G28" s="40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H28" s="41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J28" s="41" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K28" s="40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L28" s="79">
         <v>2</v>
@@ -3117,7 +3131,7 @@
         <v>100</v>
       </c>
       <c r="O28" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P28" s="53">
         <v>1.2999999999999999E-3</v>
@@ -3135,31 +3149,31 @@
         <v>20</v>
       </c>
       <c r="C29" s="63" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D29" s="38" t="s">
         <v>27</v>
       </c>
       <c r="E29" s="38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G29" s="67" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K29" s="38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L29" s="78">
         <v>2</v>
@@ -3172,7 +3186,7 @@
         <v>50</v>
       </c>
       <c r="O29" s="74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P29" s="52">
         <v>2.7000000000000001E-3</v>
@@ -3190,31 +3204,31 @@
         <v>21</v>
       </c>
       <c r="C30" s="64" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D30" s="40" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F30" s="41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G30" s="40" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H30" s="41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J30" s="41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K30" s="40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L30" s="79">
         <v>2</v>
@@ -3227,7 +3241,7 @@
         <v>100</v>
       </c>
       <c r="O30" s="73" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P30" s="53">
         <v>8.9999999999999998E-4</v>
@@ -3245,31 +3259,31 @@
         <v>22</v>
       </c>
       <c r="C31" s="66" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D31" s="67" t="s">
         <v>29</v>
       </c>
       <c r="E31" s="67" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F31" s="68" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G31" s="67" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H31" s="68" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I31" s="67" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J31" s="68" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K31" s="67" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L31" s="80">
         <v>8</v>
@@ -3282,13 +3296,13 @@
         <v>160</v>
       </c>
       <c r="O31" s="75" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P31" s="69" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q31" s="70" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="R31" s="67"/>
     </row>
@@ -3299,31 +3313,31 @@
         <v>23</v>
       </c>
       <c r="C32" s="64" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D32" s="40" t="s">
         <v>30</v>
       </c>
       <c r="E32" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F32" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G32" s="40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H32" s="41" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J32" s="41" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K32" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L32" s="79">
         <v>1</v>
@@ -3336,7 +3350,7 @@
         <v>30</v>
       </c>
       <c r="O32" s="72" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P32" s="53">
         <v>4.1399999999999999E-2</v>
@@ -3354,31 +3368,31 @@
         <v>24</v>
       </c>
       <c r="C33" s="63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D33" s="38" t="s">
         <v>31</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G33" s="67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J33" s="39" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K33" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L33" s="78">
         <v>1</v>
@@ -3391,7 +3405,7 @@
         <v>22</v>
       </c>
       <c r="O33" s="71" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P33" s="52">
         <v>10.652799999999999</v>
@@ -3401,7 +3415,7 @@
         <v>234.36159999999998</v>
       </c>
       <c r="R33" s="99" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -3411,31 +3425,31 @@
         <v>25</v>
       </c>
       <c r="C34" s="64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D34" s="40" t="s">
         <v>32</v>
       </c>
       <c r="E34" s="40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F34" s="41" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G34" s="77" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H34" s="41" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I34" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J34" s="41" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K34" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L34" s="79">
         <v>1</v>
@@ -3448,7 +3462,7 @@
         <v>22</v>
       </c>
       <c r="O34" s="72" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P34" s="53">
         <v>1.6387</v>
@@ -3466,31 +3480,31 @@
         <v>26</v>
       </c>
       <c r="C35" s="63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D35" s="38" t="s">
         <v>33</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G35" s="67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J35" s="39" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K35" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L35" s="78">
         <v>1</v>
@@ -3503,7 +3517,7 @@
         <v>22</v>
       </c>
       <c r="O35" s="71" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P35" s="52">
         <v>3.0720999999999998</v>
@@ -3521,31 +3535,31 @@
         <v>27</v>
       </c>
       <c r="C36" s="64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D36" s="40" t="s">
         <v>34</v>
       </c>
       <c r="E36" s="40" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F36" s="41" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G36" s="76" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H36" s="41" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I36" s="40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J36" s="41" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K36" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L36" s="79">
         <v>1</v>
@@ -3558,7 +3572,7 @@
         <v>22</v>
       </c>
       <c r="O36" s="72" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P36" s="53">
         <v>1.8360000000000001</v>
@@ -3576,31 +3590,31 @@
         <v>28</v>
       </c>
       <c r="C37" s="63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D37" s="38" t="s">
         <v>35</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G37" s="38" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K37" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L37" s="78">
         <v>1</v>
@@ -3613,7 +3627,7 @@
         <v>25</v>
       </c>
       <c r="O37" s="71" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P37" s="52">
         <v>0.22670000000000001</v>
@@ -3631,31 +3645,31 @@
         <v>29</v>
       </c>
       <c r="C38" s="64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D38" s="40" t="s">
-        <v>36</v>
+        <v>221</v>
       </c>
       <c r="E38" s="40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F38" s="41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G38" s="40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H38" s="41" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I38" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J38" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K38" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L38" s="79">
         <v>1</v>
@@ -3668,7 +3682,7 @@
         <v>22</v>
       </c>
       <c r="O38" s="72" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P38" s="53">
         <v>1.06</v>
@@ -3686,31 +3700,31 @@
         <v>30</v>
       </c>
       <c r="C39" s="63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E39" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G39" s="38" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I39" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J39" s="39" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="K39" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="L39" s="78">
         <v>1</v>
@@ -3723,7 +3737,7 @@
         <v>22</v>
       </c>
       <c r="O39" s="71" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P39" s="52">
         <v>0.53300000000000003</v>
@@ -3741,31 +3755,31 @@
         <v>31</v>
       </c>
       <c r="C40" s="64" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D40" s="40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E40" s="40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F40" s="41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G40" s="40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H40" s="41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I40" s="40" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J40" s="41" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K40" s="40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L40" s="79">
         <v>1</v>
@@ -3778,7 +3792,7 @@
         <v>22</v>
       </c>
       <c r="O40" s="72" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="P40" s="53">
         <v>0.505</v>
@@ -3796,31 +3810,31 @@
         <v>32</v>
       </c>
       <c r="C41" s="82" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D41" s="62" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E41" s="62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F41" s="83" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G41" s="62" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H41" s="83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I41" s="62" t="s">
+        <v>176</v>
+      </c>
+      <c r="J41" s="83" t="s">
+        <v>176</v>
+      </c>
+      <c r="K41" s="62" t="s">
         <v>177</v>
-      </c>
-      <c r="J41" s="83" t="s">
-        <v>177</v>
-      </c>
-      <c r="K41" s="62" t="s">
-        <v>178</v>
       </c>
       <c r="L41" s="84">
         <v>1</v>
@@ -3833,7 +3847,7 @@
         <v>22</v>
       </c>
       <c r="O41" s="71" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="P41" s="52">
         <v>0.69</v>
@@ -3903,37 +3917,37 @@
     <mergeCell ref="N43:P43"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1"/>
-    <hyperlink ref="O11" r:id="rId2"/>
-    <hyperlink ref="O12" r:id="rId3"/>
-    <hyperlink ref="O13" r:id="rId4"/>
-    <hyperlink ref="O14" r:id="rId5"/>
-    <hyperlink ref="O15" r:id="rId6"/>
-    <hyperlink ref="O16" r:id="rId7"/>
-    <hyperlink ref="O17" r:id="rId8"/>
-    <hyperlink ref="O18" r:id="rId9"/>
-    <hyperlink ref="O19" r:id="rId10"/>
-    <hyperlink ref="O20" r:id="rId11"/>
-    <hyperlink ref="O21" r:id="rId12"/>
-    <hyperlink ref="O22" r:id="rId13"/>
-    <hyperlink ref="O23" r:id="rId14"/>
-    <hyperlink ref="O24" r:id="rId15"/>
-    <hyperlink ref="O25" r:id="rId16"/>
-    <hyperlink ref="O26" r:id="rId17"/>
-    <hyperlink ref="O27" r:id="rId18"/>
-    <hyperlink ref="O28" r:id="rId19"/>
-    <hyperlink ref="O29" r:id="rId20"/>
-    <hyperlink ref="O32" r:id="rId21"/>
-    <hyperlink ref="O33" r:id="rId22"/>
-    <hyperlink ref="O34" r:id="rId23"/>
-    <hyperlink ref="O35" r:id="rId24"/>
-    <hyperlink ref="O36" r:id="rId25"/>
-    <hyperlink ref="O37" r:id="rId26"/>
-    <hyperlink ref="O39" r:id="rId27"/>
-    <hyperlink ref="O41" r:id="rId28"/>
-    <hyperlink ref="O30" r:id="rId29"/>
-    <hyperlink ref="O38" r:id="rId30"/>
-    <hyperlink ref="O40" r:id="rId31"/>
+    <hyperlink ref="O10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="O11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="O12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="O13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="O14" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="O15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="O16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="O17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="O18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="O19" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="O20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="O21" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="O22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="O23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="O25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="O26" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="O27" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="O28" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="O29" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="O32" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="O33" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="O34" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="O35" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="O36" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="O37" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="O39" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="O41" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="O30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="O38" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="O40" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>

</xml_diff>